<commit_message>
feat: support per-device Modbus slave roles and alarm point sheets
</commit_message>
<xml_diff>
--- a/docs/pointsheet-template-example.xlsx
+++ b/docs/pointsheet-template-example.xlsx
@@ -6,13 +6,14 @@
   <sheets>
     <sheet sheetId="1" name="设备信息" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="SYS" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="告警规则" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="42">
   <si>
     <t>key</t>
   </si>
@@ -20,6 +21,12 @@
     <t>value</t>
   </si>
   <si>
+    <t>点位表版本</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
     <t>设备名</t>
   </si>
   <si>
@@ -80,6 +87,12 @@
     <t>枚举</t>
   </si>
   <si>
+    <t>小数位数</t>
+  </si>
+  <si>
+    <t>告警数量</t>
+  </si>
+  <si>
     <t>加热器温度</t>
   </si>
   <si>
@@ -105,13 +118,34 @@
   </si>
   <si>
     <t>0=OFF;1=ON</t>
+  </si>
+  <si>
+    <t>告警条件</t>
+  </si>
+  <si>
+    <t>原始值阈值</t>
+  </si>
+  <si>
+    <t>告警提示</t>
+  </si>
+  <si>
+    <t>&gt;=</t>
+  </si>
+  <si>
+    <t>温度过高</t>
+  </si>
+  <si>
+    <t>&lt;</t>
+  </si>
+  <si>
+    <t>温度过低</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -119,13 +153,22 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF303030"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -140,8 +183,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -481,59 +530,67 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="44" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B6" t="s">
-        <v>7</v>
+      <c r="B6" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -544,160 +601,268 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="32" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="11" width="12" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2">
+    <row r="1" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="2">
+        <v>3</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="2">
+        <v>0</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" s="2">
+        <v>3</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0</v>
+      </c>
+      <c r="I5" s="2">
+        <v>1</v>
+      </c>
+      <c r="J5" s="2">
+        <v>1</v>
+      </c>
+      <c r="K5" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="2">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2">
+        <v>0</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" s="2">
+        <v>3</v>
+      </c>
+      <c r="H6" s="2">
+        <v>1</v>
+      </c>
+      <c r="I6" s="2">
+        <v>1</v>
+      </c>
+      <c r="J6" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="2">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2">
+        <v>0</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7" s="2">
+        <v>3</v>
+      </c>
+      <c r="H7" s="2">
+        <v>2</v>
+      </c>
+      <c r="I7" s="2">
+        <v>1</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:K4"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="48" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D2">
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="2">
         <v>3</v>
       </c>
-      <c r="E2" t="s">
+      <c r="C2" s="2">
+        <v>0</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E2" s="2">
+        <v>800</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5">
-        <v>0.1</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G5">
+      <c r="B3" s="2">
         <v>3</v>
       </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G6">
-        <v>3</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7" t="s">
-        <v>30</v>
-      </c>
-      <c r="G7">
-        <v>3</v>
-      </c>
-      <c r="H7">
-        <v>2</v>
-      </c>
-      <c r="I7">
-        <v>1</v>
+      <c r="C3" s="2">
+        <v>0</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>